<commit_message>
Fixing pdf rendering issue, was comming from kableExtra package.
</commit_message>
<xml_diff>
--- a/Input/Parameters.GSA.xlsx
+++ b/Input/Parameters.GSA.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="7" documentId="8_{9F8F1050-7464-48FE-993A-42AA76CDA599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84242BAB-96E2-4426-BD0A-56BA4EADC417}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8B755656-890E-4004-B586-F26C217A2676}"/>
+    <workbookView minimized="1" xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8210" xr2:uid="{8B755656-890E-4004-B586-F26C217A2676}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters.GSA" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Parameters.GSA!$A$1:$O$53</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1439,9 +1452,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE34F6B3-7424-4572-8CEB-2855C0B6D4A8}">
   <dimension ref="A1:O53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1488,7 +1501,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1535,7 +1548,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1582,7 +1595,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1629,7 +1642,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1676,7 +1689,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1723,7 +1736,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1770,7 +1783,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1817,7 +1830,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -1864,7 +1877,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -1911,7 +1924,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -1958,7 +1971,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -2005,7 +2018,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>57</v>
       </c>
@@ -2052,7 +2065,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -2099,7 +2112,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>64</v>
       </c>
@@ -2146,7 +2159,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -2193,7 +2206,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -2240,7 +2253,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>72</v>
       </c>
@@ -2287,7 +2300,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>74</v>
       </c>
@@ -2334,7 +2347,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>76</v>
       </c>
@@ -2381,7 +2394,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>78</v>
       </c>
@@ -2428,7 +2441,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>80</v>
       </c>
@@ -2475,7 +2488,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>82</v>
       </c>
@@ -2522,7 +2535,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>84</v>
       </c>
@@ -2569,7 +2582,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>86</v>
       </c>
@@ -2616,7 +2629,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -2663,7 +2676,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>91</v>
       </c>
@@ -2710,7 +2723,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>95</v>
       </c>
@@ -2757,7 +2770,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>100</v>
       </c>
@@ -2804,7 +2817,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -2851,7 +2864,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>107</v>
       </c>
@@ -2898,7 +2911,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>111</v>
       </c>
@@ -2945,7 +2958,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>115</v>
       </c>
@@ -2992,7 +3005,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>120</v>
       </c>
@@ -3039,7 +3052,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>122</v>
       </c>
@@ -3086,7 +3099,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>124</v>
       </c>
@@ -3133,7 +3146,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>126</v>
       </c>
@@ -3180,7 +3193,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>128</v>
       </c>
@@ -3227,7 +3240,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>130</v>
       </c>
@@ -3274,7 +3287,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>135</v>
       </c>
@@ -3321,7 +3334,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>140</v>
       </c>
@@ -3368,7 +3381,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>144</v>
       </c>
@@ -3415,7 +3428,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>147</v>
       </c>
@@ -3462,7 +3475,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>150</v>
       </c>
@@ -3509,7 +3522,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>154</v>
       </c>
@@ -3556,7 +3569,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>158</v>
       </c>
@@ -3603,7 +3616,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>162</v>
       </c>
@@ -3650,7 +3663,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>165</v>
       </c>
@@ -3697,7 +3710,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>168</v>
       </c>
@@ -3744,7 +3757,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>171</v>
       </c>
@@ -3791,7 +3804,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>173</v>
       </c>
@@ -3835,7 +3848,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>176</v>
       </c>
@@ -3882,7 +3895,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>179</v>
       </c>
@@ -3936,6 +3949,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002AA8BEAC825CAE4DA772B4C276EF423C" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="4363adfface29496c4692934bfc386e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="568ff3df-f16a-482d-bb3c-58af1efa1658" xmlns:ns3="13cea704-446d-46be-be94-9e10425fef80" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5ef7a87983d964890dd86635184f037c" ns2:_="" ns3:_="">
     <xsd:import namespace="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
@@ -4146,15 +4168,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4166,13 +4179,38 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E94BB32-A682-4CEC-BF14-2FD400D8CB25}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{855838D0-6EC9-4E1E-A9DC-A57315143FA9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{855838D0-6EC9-4E1E-A9DC-A57315143FA9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E94BB32-A682-4CEC-BF14-2FD400D8CB25}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
+    <ds:schemaRef ds:uri="13cea704-446d-46be-be94-9e10425fef80"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70848A26-3E3F-44DC-9272-0A542831B603}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70848A26-3E3F-44DC-9272-0A542831B603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Found a unit mistake in OATP1B1 and OATP1B3 Vmax and corrected it. Added OATP2B1 absorption from intestinal lumen to intestine as with the previous change the model was under predicting absorption.
</commit_message>
<xml_diff>
--- a/Input/Parameters.GSA.xlsx
+++ b/Input/Parameters.GSA.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4.sharepoint.com/sites/PARCProjectChrysanthi-CChannel/Gedeelde documenten/C_Channel/CP_L_R/PARC_PFOA_mechanistic/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{9F8F1050-7464-48FE-993A-42AA76CDA599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84242BAB-96E2-4426-BD0A-56BA4EADC417}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{9F8F1050-7464-48FE-993A-42AA76CDA599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{075961D8-6322-49A4-AC9E-D3D823F8071C}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8210" xr2:uid="{8B755656-890E-4004-B586-F26C217A2676}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8B755656-890E-4004-B586-F26C217A2676}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters.GSA" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Parameters.GSA!$A$1:$O$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$A$1:$K$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="184">
   <si>
     <t>Parameter</t>
   </si>
@@ -161,9 +163,6 @@
     <t>Surface area of the small intestine</t>
   </si>
   <si>
-    <t>SA_SI</t>
-  </si>
-  <si>
     <t>cm2</t>
   </si>
   <si>
@@ -353,9 +352,6 @@
     <t>Plasma to liver albumin concentration ratio</t>
   </si>
   <si>
-    <t>R_L_ic</t>
-  </si>
-  <si>
     <t>Utsey et al. 2020 https://doi.org/10.1124/dmd.120.090498</t>
   </si>
   <si>
@@ -569,18 +565,12 @@
     <t>Time to stop the exposure</t>
   </si>
   <si>
-    <t>EXP_STOP</t>
-  </si>
-  <si>
     <t>day</t>
   </si>
   <si>
     <t xml:space="preserve">Oral concentration </t>
   </si>
   <si>
-    <t>COral</t>
-  </si>
-  <si>
     <t>ug/kg/day</t>
   </si>
   <si>
@@ -588,12 +578,30 @@
   </si>
   <si>
     <t>Upper and lower limits taken from table 22 page 148</t>
+  </si>
+  <si>
+    <t>R_L_ec</t>
+  </si>
+  <si>
+    <t>expOral</t>
+  </si>
+  <si>
+    <t>expSTOP</t>
+  </si>
+  <si>
+    <t>SA_SIc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="4">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
+    <numFmt numFmtId="169" formatCode="0.0000000"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1071,11 +1079,20 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1452,9 +1469,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE34F6B3-7424-4572-8CEB-2855C0B6D4A8}">
   <dimension ref="A1:O53"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1501,7 +1523,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1548,7 +1570,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1595,7 +1617,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1642,7 +1664,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1689,7 +1711,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1736,7 +1758,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1783,15 +1805,15 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" t="s">
         <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>42</v>
       </c>
       <c r="D8" s="1">
         <v>60500</v>
@@ -1806,7 +1828,7 @@
         <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I8" s="1">
         <v>50000</v>
@@ -1824,18 +1846,18 @@
         <v>5</v>
       </c>
       <c r="N8" t="s">
+        <v>43</v>
+      </c>
+      <c r="O8" t="s">
         <v>44</v>
       </c>
-      <c r="O8" t="s">
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>46</v>
-      </c>
-      <c r="B9" t="s">
-        <v>47</v>
       </c>
       <c r="C9" t="s">
         <v>18</v>
@@ -1877,12 +1899,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s">
         <v>48</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
@@ -1918,18 +1940,18 @@
         <v>4</v>
       </c>
       <c r="N10" t="s">
+        <v>49</v>
+      </c>
+      <c r="O10" t="s">
         <v>50</v>
       </c>
-      <c r="O10" t="s">
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>52</v>
-      </c>
-      <c r="B11" t="s">
-        <v>53</v>
       </c>
       <c r="C11" t="s">
         <v>18</v>
@@ -1965,18 +1987,18 @@
         <v>4</v>
       </c>
       <c r="N11" t="s">
+        <v>53</v>
+      </c>
+      <c r="O11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>54</v>
       </c>
-      <c r="O11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>55</v>
-      </c>
-      <c r="B12" t="s">
-        <v>56</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -2018,12 +2040,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
         <v>57</v>
-      </c>
-      <c r="B13" t="s">
-        <v>58</v>
       </c>
       <c r="C13" t="s">
         <v>18</v>
@@ -2059,18 +2081,18 @@
         <v>4</v>
       </c>
       <c r="N13" t="s">
+        <v>58</v>
+      </c>
+      <c r="O13" t="s">
         <v>59</v>
       </c>
-      <c r="O13" t="s">
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>61</v>
-      </c>
-      <c r="B14" t="s">
-        <v>62</v>
       </c>
       <c r="C14" t="s">
         <v>18</v>
@@ -2106,18 +2128,18 @@
         <v>4</v>
       </c>
       <c r="N14" t="s">
+        <v>62</v>
+      </c>
+      <c r="O14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>63</v>
       </c>
-      <c r="O14" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>64</v>
-      </c>
-      <c r="B15" t="s">
-        <v>65</v>
       </c>
       <c r="C15" t="s">
         <v>18</v>
@@ -2153,18 +2175,18 @@
         <v>4</v>
       </c>
       <c r="N15" t="s">
+        <v>65</v>
+      </c>
+      <c r="O15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>66</v>
       </c>
-      <c r="O15" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>67</v>
-      </c>
-      <c r="B16" t="s">
-        <v>68</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
@@ -2200,18 +2222,18 @@
         <v>4</v>
       </c>
       <c r="N16" t="s">
+        <v>68</v>
+      </c>
+      <c r="O16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>69</v>
       </c>
-      <c r="O16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>70</v>
-      </c>
-      <c r="B17" t="s">
-        <v>71</v>
       </c>
       <c r="C17" t="s">
         <v>18</v>
@@ -2253,12 +2275,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
         <v>72</v>
-      </c>
-      <c r="B18" t="s">
-        <v>73</v>
       </c>
       <c r="C18" t="s">
         <v>18</v>
@@ -2300,12 +2322,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" t="s">
         <v>74</v>
-      </c>
-      <c r="B19" t="s">
-        <v>75</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -2347,12 +2369,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
         <v>76</v>
-      </c>
-      <c r="B20" t="s">
-        <v>77</v>
       </c>
       <c r="C20" t="s">
         <v>18</v>
@@ -2394,12 +2416,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" t="s">
         <v>78</v>
-      </c>
-      <c r="B21" t="s">
-        <v>79</v>
       </c>
       <c r="C21" t="s">
         <v>18</v>
@@ -2441,12 +2463,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" t="s">
         <v>80</v>
-      </c>
-      <c r="B22" t="s">
-        <v>81</v>
       </c>
       <c r="C22" t="s">
         <v>18</v>
@@ -2488,12 +2510,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" t="s">
         <v>82</v>
-      </c>
-      <c r="B23" t="s">
-        <v>83</v>
       </c>
       <c r="C23" t="s">
         <v>18</v>
@@ -2535,12 +2557,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" t="s">
         <v>84</v>
-      </c>
-      <c r="B24" t="s">
-        <v>85</v>
       </c>
       <c r="C24" t="s">
         <v>18</v>
@@ -2582,12 +2604,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" t="s">
         <v>86</v>
-      </c>
-      <c r="B25" t="s">
-        <v>87</v>
       </c>
       <c r="C25" t="s">
         <v>18</v>
@@ -2626,15 +2648,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
         <v>89</v>
-      </c>
-      <c r="B26" t="s">
-        <v>90</v>
       </c>
       <c r="C26" t="s">
         <v>18</v>
@@ -2652,7 +2674,7 @@
         <v>19</v>
       </c>
       <c r="H26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I26" s="1">
         <v>0.14899999999999999</v>
@@ -2676,12 +2698,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" t="s">
         <v>91</v>
-      </c>
-      <c r="B27" t="s">
-        <v>92</v>
       </c>
       <c r="C27" t="s">
         <v>25</v>
@@ -2699,7 +2721,7 @@
         <v>19</v>
       </c>
       <c r="H27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I27" s="1">
         <v>43.2</v>
@@ -2717,21 +2739,21 @@
         <v>5</v>
       </c>
       <c r="N27" t="s">
+        <v>92</v>
+      </c>
+      <c r="O27" t="s">
         <v>93</v>
       </c>
-      <c r="O27" t="s">
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
         <v>95</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>96</v>
-      </c>
-      <c r="C28" t="s">
-        <v>97</v>
       </c>
       <c r="D28" s="1">
         <v>3.36</v>
@@ -2764,18 +2786,18 @@
         <v>3</v>
       </c>
       <c r="N28" t="s">
+        <v>97</v>
+      </c>
+      <c r="O28" t="s">
         <v>98</v>
       </c>
-      <c r="O28" t="s">
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
         <v>100</v>
-      </c>
-      <c r="B29" t="s">
-        <v>101</v>
       </c>
       <c r="C29" t="s">
         <v>18</v>
@@ -2811,18 +2833,18 @@
         <v>3</v>
       </c>
       <c r="N29" t="s">
+        <v>101</v>
+      </c>
+      <c r="O29" t="s">
         <v>102</v>
       </c>
-      <c r="O29" t="s">
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>104</v>
-      </c>
       <c r="B30" t="s">
-        <v>105</v>
+        <v>180</v>
       </c>
       <c r="C30" t="s">
         <v>18</v>
@@ -2858,18 +2880,18 @@
         <v>3</v>
       </c>
       <c r="N30" t="s">
+        <v>104</v>
+      </c>
+      <c r="O30" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" t="s">
         <v>106</v>
-      </c>
-      <c r="O30" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>107</v>
-      </c>
-      <c r="B31" t="s">
-        <v>108</v>
       </c>
       <c r="C31" t="s">
         <v>18</v>
@@ -2905,18 +2927,18 @@
         <v>4</v>
       </c>
       <c r="N31" t="s">
+        <v>107</v>
+      </c>
+      <c r="O31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>109</v>
       </c>
-      <c r="O31" t="s">
+      <c r="B32" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>111</v>
-      </c>
-      <c r="B32" t="s">
-        <v>112</v>
       </c>
       <c r="C32" t="s">
         <v>18</v>
@@ -2952,18 +2974,18 @@
         <v>3</v>
       </c>
       <c r="N32" t="s">
+        <v>111</v>
+      </c>
+      <c r="O32" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>113</v>
       </c>
-      <c r="O32" t="s">
+      <c r="B33" t="s">
         <v>114</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>115</v>
-      </c>
-      <c r="B33" t="s">
-        <v>116</v>
       </c>
       <c r="C33" t="s">
         <v>18</v>
@@ -2978,7 +3000,7 @@
         <v>18</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H33" t="s">
         <v>20</v>
@@ -2999,18 +3021,18 @@
         <v>18</v>
       </c>
       <c r="N33" t="s">
+        <v>116</v>
+      </c>
+      <c r="O33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>118</v>
       </c>
-      <c r="O33" t="s">
+      <c r="B34" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>120</v>
-      </c>
-      <c r="B34" t="s">
-        <v>121</v>
       </c>
       <c r="C34" t="s">
         <v>18</v>
@@ -3025,7 +3047,7 @@
         <v>18</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H34" t="s">
         <v>20</v>
@@ -3046,18 +3068,18 @@
         <v>18</v>
       </c>
       <c r="N34" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O34" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B35" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s">
         <v>18</v>
@@ -3072,7 +3094,7 @@
         <v>18</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H35" t="s">
         <v>20</v>
@@ -3093,18 +3115,18 @@
         <v>18</v>
       </c>
       <c r="N35" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O35" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C36" t="s">
         <v>18</v>
@@ -3119,7 +3141,7 @@
         <v>18</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H36" t="s">
         <v>20</v>
@@ -3140,18 +3162,18 @@
         <v>18</v>
       </c>
       <c r="N36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O36" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B37" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C37" t="s">
         <v>18</v>
@@ -3166,7 +3188,7 @@
         <v>18</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H37" t="s">
         <v>20</v>
@@ -3187,18 +3209,18 @@
         <v>18</v>
       </c>
       <c r="N37" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O37" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C38" t="s">
         <v>18</v>
@@ -3213,7 +3235,7 @@
         <v>18</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H38" t="s">
         <v>20</v>
@@ -3234,21 +3256,21 @@
         <v>18</v>
       </c>
       <c r="N38" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O38" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B39" t="s">
+        <v>129</v>
+      </c>
+      <c r="C39" t="s">
         <v>130</v>
-      </c>
-      <c r="B39" t="s">
-        <v>131</v>
-      </c>
-      <c r="C39" t="s">
-        <v>132</v>
       </c>
       <c r="D39" s="1">
         <v>7.3100000000000003E-6</v>
@@ -3281,21 +3303,21 @@
         <v>4</v>
       </c>
       <c r="N39" t="s">
+        <v>131</v>
+      </c>
+      <c r="O39" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>133</v>
       </c>
-      <c r="O39" t="s">
+      <c r="B40" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="C40" t="s">
         <v>135</v>
-      </c>
-      <c r="B40" t="s">
-        <v>136</v>
-      </c>
-      <c r="C40" t="s">
-        <v>137</v>
       </c>
       <c r="D40" s="1">
         <v>2.3099999999999999E-6</v>
@@ -3307,7 +3329,7 @@
         <v>0.13</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H40" t="s">
         <v>20</v>
@@ -3328,21 +3350,21 @@
         <v>18</v>
       </c>
       <c r="N40" t="s">
+        <v>136</v>
+      </c>
+      <c r="O40" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>138</v>
       </c>
-      <c r="O40" t="s">
+      <c r="B41" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="C41" t="s">
         <v>140</v>
-      </c>
-      <c r="B41" t="s">
-        <v>141</v>
-      </c>
-      <c r="C41" t="s">
-        <v>142</v>
       </c>
       <c r="D41" s="1">
         <v>52.7</v>
@@ -3375,21 +3397,21 @@
         <v>3</v>
       </c>
       <c r="N41" t="s">
+        <v>141</v>
+      </c>
+      <c r="O41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>142</v>
+      </c>
+      <c r="B42" t="s">
         <v>143</v>
       </c>
-      <c r="O41" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>144</v>
-      </c>
-      <c r="B42" t="s">
-        <v>145</v>
-      </c>
       <c r="C42" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D42" s="1">
         <v>2.6900000000000001E-6</v>
@@ -3401,7 +3423,7 @@
         <v>0.17</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H42" t="s">
         <v>20</v>
@@ -3422,21 +3444,21 @@
         <v>18</v>
       </c>
       <c r="N42" t="s">
+        <v>144</v>
+      </c>
+      <c r="O42" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" t="s">
         <v>146</v>
       </c>
-      <c r="O42" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>147</v>
-      </c>
-      <c r="B43" t="s">
-        <v>148</v>
-      </c>
       <c r="C43" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D43" s="1">
         <v>91.6</v>
@@ -3469,18 +3491,18 @@
         <v>3</v>
       </c>
       <c r="N43" t="s">
+        <v>147</v>
+      </c>
+      <c r="O43" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>148</v>
+      </c>
+      <c r="B44" t="s">
         <v>149</v>
-      </c>
-      <c r="O43" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>150</v>
-      </c>
-      <c r="B44" t="s">
-        <v>151</v>
       </c>
       <c r="C44" t="s">
         <v>18</v>
@@ -3495,10 +3517,10 @@
         <v>18</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I44" s="1">
         <v>1</v>
@@ -3516,18 +3538,18 @@
         <v>18</v>
       </c>
       <c r="N44" t="s">
+        <v>150</v>
+      </c>
+      <c r="O44" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>152</v>
       </c>
-      <c r="O44" t="s">
+      <c r="B45" t="s">
         <v>153</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" t="s">
-        <v>155</v>
       </c>
       <c r="C45" t="s">
         <v>18</v>
@@ -3542,10 +3564,10 @@
         <v>18</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I45" s="1">
         <v>1</v>
@@ -3563,21 +3585,21 @@
         <v>18</v>
       </c>
       <c r="N45" t="s">
+        <v>154</v>
+      </c>
+      <c r="O45" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>156</v>
       </c>
-      <c r="O45" t="s">
+      <c r="B46" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="C46" t="s">
         <v>158</v>
-      </c>
-      <c r="B46" t="s">
-        <v>159</v>
-      </c>
-      <c r="C46" t="s">
-        <v>160</v>
       </c>
       <c r="D46" s="1">
         <v>7.1</v>
@@ -3589,10 +3611,10 @@
         <v>0.18</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I46" s="1">
         <v>4.8899999999999997</v>
@@ -3610,21 +3632,21 @@
         <v>18</v>
       </c>
       <c r="N46" t="s">
+        <v>159</v>
+      </c>
+      <c r="O46" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>160</v>
+      </c>
+      <c r="B47" t="s">
         <v>161</v>
       </c>
-      <c r="O46" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>162</v>
-      </c>
-      <c r="B47" t="s">
-        <v>163</v>
-      </c>
       <c r="C47" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D47" s="1">
         <v>16.399999999999999</v>
@@ -3657,18 +3679,18 @@
         <v>3</v>
       </c>
       <c r="N47" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="O47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B48" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C48" t="s">
         <v>18</v>
@@ -3683,10 +3705,10 @@
         <v>18</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I48" s="1">
         <v>1</v>
@@ -3704,21 +3726,21 @@
         <v>18</v>
       </c>
       <c r="N48" t="s">
+        <v>165</v>
+      </c>
+      <c r="O48" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>166</v>
+      </c>
+      <c r="B49" t="s">
         <v>167</v>
       </c>
-      <c r="O48" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>168</v>
-      </c>
-      <c r="B49" t="s">
-        <v>169</v>
-      </c>
       <c r="C49" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D49" s="1">
         <v>4.4999999999999997E-3</v>
@@ -3730,10 +3752,10 @@
         <v>0.11</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I49" s="1">
         <v>3.63E-3</v>
@@ -3751,21 +3773,21 @@
         <v>18</v>
       </c>
       <c r="N49" t="s">
+        <v>168</v>
+      </c>
+      <c r="O49" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>169</v>
+      </c>
+      <c r="B50" t="s">
         <v>170</v>
       </c>
-      <c r="O49" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>171</v>
-      </c>
-      <c r="B50" t="s">
-        <v>172</v>
-      </c>
       <c r="C50" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D50" s="1">
         <v>47</v>
@@ -3798,18 +3820,18 @@
         <v>3</v>
       </c>
       <c r="N50" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O50" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B51" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C51" t="s">
         <v>18</v>
@@ -3824,10 +3846,10 @@
         <v>18</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H51" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I51" s="1">
         <v>1</v>
@@ -3845,18 +3867,18 @@
         <v>18</v>
       </c>
       <c r="N51" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>174</v>
+      </c>
+      <c r="B52" t="s">
+        <v>182</v>
+      </c>
+      <c r="C52" t="s">
         <v>175</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>176</v>
-      </c>
-      <c r="B52" t="s">
-        <v>177</v>
-      </c>
-      <c r="C52" t="s">
-        <v>178</v>
       </c>
       <c r="D52" s="1">
         <v>18300</v>
@@ -3868,7 +3890,7 @@
         <v>18</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H52" t="s">
         <v>32</v>
@@ -3895,15 +3917,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B53" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C53" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D53" s="1">
         <v>4.8000000000000001E-2</v>
@@ -3915,7 +3937,7 @@
         <v>18</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H53" t="s">
         <v>32</v>
@@ -3936,14 +3958,1887 @@
         <v>18</v>
       </c>
       <c r="N53" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="O53" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O53" xr:uid="{CE34F6B3-7424-4572-8CEB-2855C0B6D4A8}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F2D757-9DD9-49EE-B2A1-1E86CE6FF1DD}">
+  <dimension ref="A1:K56"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="4">
+        <v>74.2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>61.3</v>
+      </c>
+      <c r="E2" s="4">
+        <v>87</v>
+      </c>
+      <c r="F2" s="4">
+        <v>74.2</v>
+      </c>
+      <c r="G2" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H2" s="4">
+        <v>4</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4">
+        <v>5230</v>
+      </c>
+      <c r="D3" s="4">
+        <v>4330</v>
+      </c>
+      <c r="E3" s="4">
+        <v>6140</v>
+      </c>
+      <c r="F3" s="4">
+        <v>5230</v>
+      </c>
+      <c r="G3" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H3" s="4">
+        <v>4</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.42699999999999999</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.501</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.42699999999999999</v>
+      </c>
+      <c r="G4" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H4" s="4">
+        <v>4</v>
+      </c>
+      <c r="I4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>4.07E-2</v>
+      </c>
+      <c r="E5" s="4">
+        <v>4.9700000000000001E-2</v>
+      </c>
+      <c r="F5" s="4">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="G5" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H5" s="4">
+        <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="8">
+        <v>1.4E-2</v>
+      </c>
+      <c r="D6" s="8">
+        <v>1.26E-2</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1.54E-2</v>
+      </c>
+      <c r="F6" s="8">
+        <v>1.4E-2</v>
+      </c>
+      <c r="G6" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H6" s="8">
+        <v>2</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="8">
+        <v>2.3800000000000002E-2</v>
+      </c>
+      <c r="D7" s="8">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1.83</v>
+      </c>
+      <c r="F7" s="8">
+        <v>2.3800000000000002E-2</v>
+      </c>
+      <c r="G7" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H7" s="8">
+        <v>4</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="8">
+        <v>60500</v>
+      </c>
+      <c r="D8" s="8">
+        <v>50000</v>
+      </c>
+      <c r="E8" s="8">
+        <v>71000</v>
+      </c>
+      <c r="F8" s="8">
+        <v>60500</v>
+      </c>
+      <c r="G8" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H8" s="8">
+        <v>5</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="8">
+        <v>2.47E-2</v>
+      </c>
+      <c r="D9" s="9">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="E9" s="9">
+        <v>2.7199999999999998E-2</v>
+      </c>
+      <c r="F9" s="8">
+        <v>2.47E-2</v>
+      </c>
+      <c r="G9" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H9" s="8">
+        <v>2</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="8">
+        <v>0.57299999999999995</v>
+      </c>
+      <c r="D10" s="8">
+        <v>0.51600000000000001</v>
+      </c>
+      <c r="E10" s="8">
+        <v>0.63</v>
+      </c>
+      <c r="F10" s="8">
+        <v>0.57299999999999995</v>
+      </c>
+      <c r="G10" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H10" s="8">
+        <v>4</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="8">
+        <v>0.42699999999999999</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="E11" s="8">
+        <v>0.47</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0.42699999999999999</v>
+      </c>
+      <c r="G11" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H11" s="8">
+        <v>4</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="9">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="D12" s="8">
+        <v>3.7799999999999999E-3</v>
+      </c>
+      <c r="E12" s="8">
+        <v>4.62E-3</v>
+      </c>
+      <c r="F12" s="8">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="G12" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H12" s="8">
+        <v>4</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="8">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="D13" s="8">
+        <v>0.35799999999999998</v>
+      </c>
+      <c r="E13" s="8">
+        <v>0.438</v>
+      </c>
+      <c r="F13" s="8">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="G13" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H13" s="8">
+        <v>4</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="8">
+        <v>0.53900000000000003</v>
+      </c>
+      <c r="D14" s="8">
+        <v>0.48499999999999999</v>
+      </c>
+      <c r="E14" s="8">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="F14" s="8">
+        <v>0.53900000000000003</v>
+      </c>
+      <c r="G14" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H14" s="8">
+        <v>4</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="8">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="D15" s="8">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="E15" s="8">
+        <v>0.443</v>
+      </c>
+      <c r="F15" s="8">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="G15" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H15" s="8">
+        <v>4</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="8">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0.255</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0.311</v>
+      </c>
+      <c r="F16" s="8">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="G16" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H16" s="8">
+        <v>4</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0.247</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0.223</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="F17" s="8">
+        <v>0.247</v>
+      </c>
+      <c r="G17" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H17" s="8">
+        <v>2</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="8">
+        <v>10.3</v>
+      </c>
+      <c r="D18" s="8">
+        <v>9.23</v>
+      </c>
+      <c r="E18" s="8">
+        <v>11.3</v>
+      </c>
+      <c r="F18" s="8">
+        <v>10.3</v>
+      </c>
+      <c r="G18" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H18" s="8">
+        <v>2</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="8">
+        <v>7.6100000000000001E-2</v>
+      </c>
+      <c r="D19" s="9">
+        <v>6.8500000000000005E-2</v>
+      </c>
+      <c r="E19" s="9">
+        <v>8.3699999999999997E-2</v>
+      </c>
+      <c r="F19" s="9">
+        <v>7.6100000000000001E-2</v>
+      </c>
+      <c r="G19" s="8">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H19" s="8">
+        <v>4</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="5">
+        <v>5.1999999999999998E-2</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4.6800000000000001E-2</v>
+      </c>
+      <c r="E20" s="5">
+        <v>5.7200000000000001E-2</v>
+      </c>
+      <c r="F20" s="5">
+        <v>5.1999999999999998E-2</v>
+      </c>
+      <c r="G20" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H20" s="4">
+        <v>2</v>
+      </c>
+      <c r="I20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" t="s">
+        <v>21</v>
+      </c>
+      <c r="K20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="4">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0.13</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0.158</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="G21" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H21" s="4">
+        <v>2</v>
+      </c>
+      <c r="I21" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" t="s">
+        <v>21</v>
+      </c>
+      <c r="K21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="5">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="D22" s="5">
+        <v>5.8500000000000003E-2</v>
+      </c>
+      <c r="E22" s="5">
+        <v>7.1499999999999994E-2</v>
+      </c>
+      <c r="F22" s="5">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="G22" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H22" s="4">
+        <v>2</v>
+      </c>
+      <c r="I22" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" t="s">
+        <v>21</v>
+      </c>
+      <c r="K22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="5">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0.216</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="G23" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H23" s="4">
+        <v>4</v>
+      </c>
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="5">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="D24" s="5">
+        <v>5.79E-2</v>
+      </c>
+      <c r="E24" s="5">
+        <v>7.0699999999999999E-2</v>
+      </c>
+      <c r="F24" s="5">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="G24" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H24" s="4">
+        <v>2</v>
+      </c>
+      <c r="I24" t="s">
+        <v>18</v>
+      </c>
+      <c r="J24" t="s">
+        <v>21</v>
+      </c>
+      <c r="K24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="5">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="D25" s="5">
+        <v>1.9800000000000002E-2</v>
+      </c>
+      <c r="E25" s="5">
+        <v>2.4199999999999999E-2</v>
+      </c>
+      <c r="F25" s="5">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="G25" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H25" s="4">
+        <v>3</v>
+      </c>
+      <c r="I25" t="s">
+        <v>18</v>
+      </c>
+      <c r="J25" t="s">
+        <v>21</v>
+      </c>
+      <c r="K25" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0.21099999999999999</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="G26" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H26" s="4">
+        <v>5</v>
+      </c>
+      <c r="I26" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="4">
+        <v>62.2</v>
+      </c>
+      <c r="D27" s="4">
+        <v>43.2</v>
+      </c>
+      <c r="E27" s="4">
+        <v>120</v>
+      </c>
+      <c r="F27" s="4">
+        <v>62.2</v>
+      </c>
+      <c r="G27" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H27" s="4">
+        <v>5</v>
+      </c>
+      <c r="I27" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" t="s">
+        <v>92</v>
+      </c>
+      <c r="K27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="4">
+        <v>3.36</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3.02</v>
+      </c>
+      <c r="E28" s="4">
+        <v>3.7</v>
+      </c>
+      <c r="F28" s="4">
+        <v>3.36</v>
+      </c>
+      <c r="G28" s="4">
+        <v>9.98E-2</v>
+      </c>
+      <c r="H28" s="4">
+        <v>3</v>
+      </c>
+      <c r="I28" t="s">
+        <v>96</v>
+      </c>
+      <c r="J28" t="s">
+        <v>97</v>
+      </c>
+      <c r="K28" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="4">
+        <v>2570</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1</v>
+      </c>
+      <c r="E29" s="4">
+        <v>2880</v>
+      </c>
+      <c r="F29" s="4">
+        <v>2570</v>
+      </c>
+      <c r="G29" s="4">
+        <v>6.9900000000000004E-2</v>
+      </c>
+      <c r="H29" s="4">
+        <v>3</v>
+      </c>
+      <c r="I29" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" t="s">
+        <v>101</v>
+      </c>
+      <c r="K29" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="4">
+        <v>11.6</v>
+      </c>
+      <c r="D30" s="4">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="E30" s="4">
+        <v>13</v>
+      </c>
+      <c r="F30" s="4">
+        <v>11.6</v>
+      </c>
+      <c r="G30" s="4">
+        <v>6.9900000000000004E-2</v>
+      </c>
+      <c r="H30" s="4">
+        <v>3</v>
+      </c>
+      <c r="I30" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30" t="s">
+        <v>104</v>
+      </c>
+      <c r="K30" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="10">
+        <v>6.0999999999999997E-4</v>
+      </c>
+      <c r="D31" s="10">
+        <v>6.0999999999999999E-5</v>
+      </c>
+      <c r="E31" s="10">
+        <v>2E-3</v>
+      </c>
+      <c r="F31" s="10">
+        <v>6.0999999999999997E-4</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1</v>
+      </c>
+      <c r="H31" s="4">
+        <v>4</v>
+      </c>
+      <c r="I31" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" t="s">
+        <v>107</v>
+      </c>
+      <c r="K31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>109</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="10">
+        <v>1.89</v>
+      </c>
+      <c r="D32" s="10">
+        <v>1</v>
+      </c>
+      <c r="E32" s="10">
+        <v>3.9</v>
+      </c>
+      <c r="F32" s="10">
+        <v>1.89</v>
+      </c>
+      <c r="G32" s="4">
+        <v>0.56599999999999995</v>
+      </c>
+      <c r="H32" s="4">
+        <v>3</v>
+      </c>
+      <c r="I32" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" t="s">
+        <v>111</v>
+      </c>
+      <c r="K32" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>113</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="4">
+        <v>217</v>
+      </c>
+      <c r="D33" s="4">
+        <v>195</v>
+      </c>
+      <c r="E33" s="4">
+        <v>239</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" t="s">
+        <v>116</v>
+      </c>
+      <c r="K33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C34" s="4">
+        <v>62.8</v>
+      </c>
+      <c r="D34" s="4">
+        <v>56.5</v>
+      </c>
+      <c r="E34" s="4">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" t="s">
+        <v>116</v>
+      </c>
+      <c r="K34" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>120</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" s="4">
+        <v>134</v>
+      </c>
+      <c r="D35" s="4">
+        <v>120</v>
+      </c>
+      <c r="E35" s="4">
+        <v>147</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" t="s">
+        <v>116</v>
+      </c>
+      <c r="K35" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>122</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" s="4">
+        <v>158</v>
+      </c>
+      <c r="D36" s="4">
+        <v>142</v>
+      </c>
+      <c r="E36" s="4">
+        <v>174</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" t="s">
+        <v>116</v>
+      </c>
+      <c r="K36" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>124</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C37" s="4">
+        <v>180</v>
+      </c>
+      <c r="D37" s="4">
+        <v>162</v>
+      </c>
+      <c r="E37" s="4">
+        <v>198</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" t="s">
+        <v>116</v>
+      </c>
+      <c r="K37" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>126</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C38" s="4">
+        <v>60.9</v>
+      </c>
+      <c r="D38" s="4">
+        <v>54.8</v>
+      </c>
+      <c r="E38" s="4">
+        <v>67</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" t="s">
+        <v>18</v>
+      </c>
+      <c r="J38" t="s">
+        <v>116</v>
+      </c>
+      <c r="K38" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="12">
+        <v>7.3100000000000003E-6</v>
+      </c>
+      <c r="D39" s="12">
+        <v>6.5699999999999998E-6</v>
+      </c>
+      <c r="E39" s="12">
+        <v>8.0499999999999992E-6</v>
+      </c>
+      <c r="F39" s="4">
+        <v>7.3100000000000003E-6</v>
+      </c>
+      <c r="G39" s="4">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="H39" s="4">
+        <v>4</v>
+      </c>
+      <c r="I39" t="s">
+        <v>130</v>
+      </c>
+      <c r="J39" t="s">
+        <v>131</v>
+      </c>
+      <c r="K39" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C40" s="12">
+        <v>2.3099999999999999E-6</v>
+      </c>
+      <c r="D40" s="12">
+        <v>1.79E-6</v>
+      </c>
+      <c r="E40" s="12">
+        <v>2.8200000000000001E-6</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" t="s">
+        <v>135</v>
+      </c>
+      <c r="J40" t="s">
+        <v>136</v>
+      </c>
+      <c r="K40" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="4">
+        <v>52.7</v>
+      </c>
+      <c r="D41" s="4">
+        <v>12.3</v>
+      </c>
+      <c r="E41" s="4">
+        <v>93</v>
+      </c>
+      <c r="F41" s="4">
+        <v>52.7</v>
+      </c>
+      <c r="G41" s="4">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="H41" s="4">
+        <v>3</v>
+      </c>
+      <c r="I41" t="s">
+        <v>140</v>
+      </c>
+      <c r="J41" t="s">
+        <v>141</v>
+      </c>
+      <c r="K41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>142</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C42" s="12">
+        <v>2.6900000000000001E-6</v>
+      </c>
+      <c r="D42" s="12">
+        <v>1.88E-6</v>
+      </c>
+      <c r="E42" s="12">
+        <v>3.5099999999999999E-6</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I42" t="s">
+        <v>135</v>
+      </c>
+      <c r="J42" t="s">
+        <v>144</v>
+      </c>
+      <c r="K42" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" s="4">
+        <v>91.6</v>
+      </c>
+      <c r="D43" s="4">
+        <v>8.98</v>
+      </c>
+      <c r="E43" s="4">
+        <v>174</v>
+      </c>
+      <c r="F43" s="4">
+        <v>91.6</v>
+      </c>
+      <c r="G43" s="4">
+        <v>0.49</v>
+      </c>
+      <c r="H43" s="4">
+        <v>3</v>
+      </c>
+      <c r="I43" t="s">
+        <v>140</v>
+      </c>
+      <c r="J43" t="s">
+        <v>147</v>
+      </c>
+      <c r="K43" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>148</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="4">
+        <v>3000000</v>
+      </c>
+      <c r="D44" s="4">
+        <v>1</v>
+      </c>
+      <c r="E44" s="4">
+        <v>3300000</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" t="s">
+        <v>18</v>
+      </c>
+      <c r="J44" t="s">
+        <v>150</v>
+      </c>
+      <c r="K44" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>152</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="4">
+        <v>250000</v>
+      </c>
+      <c r="D45" s="4">
+        <v>1</v>
+      </c>
+      <c r="E45" s="4">
+        <v>275000</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" t="s">
+        <v>18</v>
+      </c>
+      <c r="J45" t="s">
+        <v>154</v>
+      </c>
+      <c r="K45" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" s="4">
+        <v>7.1</v>
+      </c>
+      <c r="D46" s="4">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="E46" s="4">
+        <v>9.31</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I46" t="s">
+        <v>158</v>
+      </c>
+      <c r="J46" t="s">
+        <v>159</v>
+      </c>
+      <c r="K46" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>160</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C47" s="4">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="D47" s="4">
+        <v>1</v>
+      </c>
+      <c r="E47" s="4">
+        <v>35.5</v>
+      </c>
+      <c r="F47" s="4">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0.61099999999999999</v>
+      </c>
+      <c r="H47" s="4">
+        <v>3</v>
+      </c>
+      <c r="I47" t="s">
+        <v>140</v>
+      </c>
+      <c r="J47" t="s">
+        <v>162</v>
+      </c>
+      <c r="K47" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>163</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C48" s="4">
+        <v>11.6</v>
+      </c>
+      <c r="D48" s="4">
+        <v>1</v>
+      </c>
+      <c r="E48" s="4">
+        <v>12.8</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I48" t="s">
+        <v>18</v>
+      </c>
+      <c r="J48" t="s">
+        <v>165</v>
+      </c>
+      <c r="K48" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>166</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="10">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="D49" s="10">
+        <v>3.63E-3</v>
+      </c>
+      <c r="E49" s="10">
+        <v>5.3699999999999998E-3</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" t="s">
+        <v>135</v>
+      </c>
+      <c r="J49" t="s">
+        <v>168</v>
+      </c>
+      <c r="K49" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>169</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C50" s="4">
+        <v>47</v>
+      </c>
+      <c r="D50" s="4">
+        <v>21</v>
+      </c>
+      <c r="E50" s="4">
+        <v>73</v>
+      </c>
+      <c r="F50" s="4">
+        <v>47</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="H50" s="4">
+        <v>3</v>
+      </c>
+      <c r="I50" t="s">
+        <v>140</v>
+      </c>
+      <c r="J50" t="s">
+        <v>168</v>
+      </c>
+      <c r="K50" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>171</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C51" s="4">
+        <v>95200</v>
+      </c>
+      <c r="D51" s="4">
+        <v>1</v>
+      </c>
+      <c r="E51" s="4">
+        <v>105000</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I51" t="s">
+        <v>18</v>
+      </c>
+      <c r="J51" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>174</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C52" s="4">
+        <v>18300</v>
+      </c>
+      <c r="D52" s="4">
+        <v>16400</v>
+      </c>
+      <c r="E52" s="4">
+        <v>20100</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I52" t="s">
+        <v>175</v>
+      </c>
+      <c r="J52" t="s">
+        <v>18</v>
+      </c>
+      <c r="K52" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>176</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C53" s="5">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="D53" s="5">
+        <v>1.2899999999999999E-3</v>
+      </c>
+      <c r="E53" s="5">
+        <v>0.22900000000000001</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I53" t="s">
+        <v>177</v>
+      </c>
+      <c r="J53" t="s">
+        <v>178</v>
+      </c>
+      <c r="K53" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D56" s="11"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K53" xr:uid="{66F2D757-9DD9-49EE-B2A1-1E86CE6FF1DD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>